<commit_message>
Regenerate dashboard with corrected SKU count
</commit_message>
<xml_diff>
--- a/Warehouse_Operations_Dashboard.xlsx
+++ b/Warehouse_Operations_Dashboard.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="📊 KPI Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="👷 Picker Productivity" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="📦 SKU Performance" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="📈 Demand Patterns" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="🚚 Delivery Cost Analysis" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="🔔 Replenishment Alerts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📊 KPI Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="👷 Picker Productivity" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📦 SKU Performance" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📈 Demand Patterns" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🚚 Delivery Cost Analysis" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔔 Replenishment Alerts" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -511,14 +511,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -542,7 +542,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -570,8 +570,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -597,8 +597,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -624,14 +624,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -655,7 +655,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -707,14 +707,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -737,7 +737,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -765,14 +765,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -795,14 +795,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -830,8 +830,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -857,8 +857,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -884,14 +884,14 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -915,7 +915,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -967,14 +967,14 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -998,7 +998,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1050,14 +1050,14 @@
 </file>
 
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1080,7 +1080,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1108,7 +1108,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -1123,9 +1123,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1145,9 +1145,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1157,7 +1157,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>12</col>
@@ -1172,9 +1172,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1184,7 +1184,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>7</col>
@@ -1199,9 +1199,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1221,9 +1221,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1233,7 +1233,7 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -1248,9 +1248,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1270,9 +1270,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1760,7 +1760,7 @@
       <c r="I11" s="10" t="n"/>
       <c r="J11" s="15" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>36</t>
         </is>
       </c>
       <c r="K11" s="8" t="n"/>

</xml_diff>